<commit_message>
feat: mejora SNA guiado y alcances temporales
</commit_message>
<xml_diff>
--- a/Scripts/diccionarios/diccionario_temas_estructurales_naucalpan.xlsx
+++ b/Scripts/diccionarios/diccionario_temas_estructurales_naucalpan.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1441"/>
+  <dimension ref="A1:D1472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26168,7 +26168,7 @@
       </c>
       <c r="B1431" t="inlineStr">
         <is>
-          <t>isaac</t>
+          <t>presidente</t>
         </is>
       </c>
       <c r="C1431" t="n">
@@ -26186,7 +26186,7 @@
       </c>
       <c r="B1432" t="inlineStr">
         <is>
-          <t>montoya</t>
+          <t>municipal</t>
         </is>
       </c>
       <c r="C1432" t="n">
@@ -26204,7 +26204,7 @@
       </c>
       <c r="B1433" t="inlineStr">
         <is>
-          <t>alcalde</t>
+          <t>gobnau</t>
         </is>
       </c>
       <c r="C1433" t="n">
@@ -26222,7 +26222,7 @@
       </c>
       <c r="B1434" t="inlineStr">
         <is>
-          <t>presidente</t>
+          <t>ciudadnaucalpan</t>
         </is>
       </c>
       <c r="C1434" t="n">
@@ -26240,7 +26240,7 @@
       </c>
       <c r="B1435" t="inlineStr">
         <is>
-          <t>municipal</t>
+          <t>ayuntamiento</t>
         </is>
       </c>
       <c r="C1435" t="n">
@@ -26258,7 +26258,7 @@
       </c>
       <c r="B1436" t="inlineStr">
         <is>
-          <t>gobnau</t>
+          <t>naucalpan</t>
         </is>
       </c>
       <c r="C1436" t="n">
@@ -26276,7 +26276,7 @@
       </c>
       <c r="B1437" t="inlineStr">
         <is>
-          <t>ciudadnaucalpan</t>
+          <t>administracion</t>
         </is>
       </c>
       <c r="C1437" t="n">
@@ -26289,12 +26289,12 @@
     <row r="1438">
       <c r="A1438" t="inlineStr">
         <is>
-          <t>Gobierno municipal</t>
+          <t>Agua</t>
         </is>
       </c>
       <c r="B1438" t="inlineStr">
         <is>
-          <t>ayuntamiento</t>
+          <t>oapas</t>
         </is>
       </c>
       <c r="C1438" t="n">
@@ -26307,55 +26307,613 @@
     <row r="1439">
       <c r="A1439" t="inlineStr">
         <is>
-          <t>Gobierno municipal</t>
+          <t>Alcalde</t>
         </is>
       </c>
       <c r="B1439" t="inlineStr">
         <is>
-          <t>naucalpan</t>
+          <t>isaac</t>
         </is>
       </c>
       <c r="C1439" t="n">
         <v>0</v>
       </c>
       <c r="D1439" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
-          <t>Gobierno municipal</t>
+          <t>Alcalde</t>
         </is>
       </c>
       <c r="B1440" t="inlineStr">
         <is>
-          <t>administracion</t>
+          <t>montoya</t>
         </is>
       </c>
       <c r="C1440" t="n">
         <v>0</v>
       </c>
       <c r="D1440" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="1441">
       <c r="A1441" t="inlineStr">
         <is>
-          <t>Agua</t>
+          <t>Alcalde</t>
         </is>
       </c>
       <c r="B1441" t="inlineStr">
         <is>
-          <t>oapas</t>
+          <t>isaacsolar</t>
         </is>
       </c>
       <c r="C1441" t="n">
         <v>0</v>
       </c>
       <c r="D1441" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>isaacmontoya</t>
+        </is>
+      </c>
+      <c r="C1442" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1442" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>isaacmontoya24</t>
+        </is>
+      </c>
+      <c r="C1443" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1443" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>isaacmontoyamarquez</t>
+        </is>
+      </c>
+      <c r="C1444" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1444" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>isaacmontoyanaucalpan</t>
+        </is>
+      </c>
+      <c r="C1445" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1445" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>isaacmartinmontoya</t>
+        </is>
+      </c>
+      <c r="C1446" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1446" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>montoyamarquez</t>
+        </is>
+      </c>
+      <c r="C1447" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1447" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>alcaldeisaac</t>
+        </is>
+      </c>
+      <c r="C1448" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1448" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>alcaldeisaacmontoya</t>
+        </is>
+      </c>
+      <c r="C1449" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1449" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>presidenteisaac</t>
+        </is>
+      </c>
+      <c r="C1450" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1450" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>presidenteisaacmontoya</t>
+        </is>
+      </c>
+      <c r="C1451" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1451" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>issac</t>
+        </is>
+      </c>
+      <c r="C1452" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1452" t="n">
         <v>0.9</v>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>isacc</t>
+        </is>
+      </c>
+      <c r="C1453" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1453" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>isac</t>
+        </is>
+      </c>
+      <c r="C1454" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1454" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>izaac</t>
+        </is>
+      </c>
+      <c r="C1455" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1455" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>momtoya</t>
+        </is>
+      </c>
+      <c r="C1456" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1456" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>montolla</t>
+        </is>
+      </c>
+      <c r="C1457" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1457" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>issamontoya</t>
+        </is>
+      </c>
+      <c r="C1458" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1458" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>issacmartinmontoya</t>
+        </is>
+      </c>
+      <c r="C1459" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1459" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>issacmontoyamarquez</t>
+        </is>
+      </c>
+      <c r="C1460" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1460" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>renunciaisaacmontoya</t>
+        </is>
+      </c>
+      <c r="C1461" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1461" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>renunciaissacmontoya</t>
+        </is>
+      </c>
+      <c r="C1462" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1462" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>fueraisaac</t>
+        </is>
+      </c>
+      <c r="C1463" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1463" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>fueraisaacmontoya</t>
+        </is>
+      </c>
+      <c r="C1464" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1464" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>alcalde</t>
+        </is>
+      </c>
+      <c r="C1465" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1465" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>edil</t>
+        </is>
+      </c>
+      <c r="C1466" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1466" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>municipe</t>
+        </is>
+      </c>
+      <c r="C1467" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1467" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>alcaldenaucalpan</t>
+        </is>
+      </c>
+      <c r="C1468" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1468" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>presidentemunicipal</t>
+        </is>
+      </c>
+      <c r="C1469" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1469" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>presidentenaucalpan</t>
+        </is>
+      </c>
+      <c r="C1470" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1470" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>presidentemunicipalnaucalpan</t>
+        </is>
+      </c>
+      <c r="C1471" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1471" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>Alcalde</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>presidentemunicipaldenaucalpan</t>
+        </is>
+      </c>
+      <c r="C1472" t="n">
+        <v>0</v>
+      </c>
+      <c r="D1472" t="n">
+        <v>0.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>